<commit_message>
Primeras pruebas: ERROR en el PREPROCESAMIENTO
</commit_message>
<xml_diff>
--- a/modelos_tfg/ResultadosCuantizacion.xlsx
+++ b/modelos_tfg/ResultadosCuantizacion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26154D92-0FBE-4B39-B41D-FED5C667143A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{889D6AC7-3FA1-41C5-B6BE-1CC0169A9FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="30" windowWidth="29040" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
   <si>
     <t>MAE</t>
   </si>
@@ -96,6 +96,9 @@
       <t>R^2</t>
     </r>
   </si>
+  <si>
+    <t>KB unroll</t>
+  </si>
 </sst>
 </file>
 
@@ -105,7 +108,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -125,6 +128,14 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -134,7 +145,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -329,31 +340,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -369,6 +381,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -649,7 +675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:I13"/>
+  <dimension ref="B3:J13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -657,173 +683,191 @@
     <col min="6" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-    </row>
-    <row r="4" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="4"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="13" t="s">
+    <row r="3" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="2"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="5" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="2:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="8" t="s">
+      <c r="J4" s="15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="8">
         <v>51.7</v>
       </c>
-      <c r="E5" s="14">
+      <c r="E5" s="10">
         <v>118.3</v>
       </c>
-      <c r="F5" s="14">
+      <c r="F5" s="10">
         <v>92.9</v>
       </c>
-      <c r="G5" s="14">
+      <c r="G5" s="10">
         <v>0.94950000000000001</v>
       </c>
-      <c r="H5" s="14">
+      <c r="H5" s="10">
         <v>0.80200000000000005</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>31.8</v>
       </c>
-    </row>
-    <row r="6" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="9"/>
-      <c r="C6" s="11" t="s">
+      <c r="J5" s="19">
+        <v>73.400000000000006</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="22"/>
+      <c r="C6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="10">
         <v>51.8</v>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="10">
         <v>118.4</v>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="10">
         <v>93</v>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="10">
         <v>0.94950000000000001</v>
       </c>
-      <c r="H6" s="14">
+      <c r="H6" s="10">
         <v>0.80210000000000004</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="3">
         <v>19.899999999999999</v>
       </c>
-    </row>
-    <row r="7" spans="2:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="1" t="s">
+      <c r="J6" s="16">
+        <v>61.6</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="8">
         <v>48.1</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="8">
         <v>125.7</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="8">
         <v>102.5</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="8">
         <v>0.93859999999999999</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="8">
         <v>0.755</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>27.7</v>
       </c>
-    </row>
-    <row r="8" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="3"/>
-      <c r="C8" s="11" t="s">
+      <c r="J7" s="19">
+        <v>79.099999999999994</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="24"/>
+      <c r="C8" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="7">
         <v>48.1</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="7">
         <v>125.6</v>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="7">
         <v>102.4</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="7">
         <v>0.93869999999999998</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="7">
         <v>0.75539999999999996</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="3">
         <v>19.8</v>
       </c>
-    </row>
-    <row r="9" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C10" s="21" t="s">
+      <c r="J8" s="16">
+        <v>71.400000000000006</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="19" t="s">
+    <row r="11" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="15">
         <v>0.1</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="14">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="20" t="s">
+    <row r="12" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="18">
         <v>0</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="12">
         <v>-1E-4</v>
       </c>
     </row>
-    <row r="13" spans="2:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="I13" s="20"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="B7:B8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Modelo LSTM predice bien
</commit_message>
<xml_diff>
--- a/modelos_tfg/ResultadosCuantizacion.xlsx
+++ b/modelos_tfg/ResultadosCuantizacion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{889D6AC7-3FA1-41C5-B6BE-1CC0169A9FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6CC97AC-7020-403D-8D76-473D66869AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="30" windowWidth="29040" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -410,6 +410,187 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>13138</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>16109</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>341586</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>133268</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{38B83F9D-7BE4-2ADC-4600-03D99AEE7A2E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="624052" y="3011557"/>
+          <a:ext cx="6733189" cy="1641159"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>6568</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>183931</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>617439</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>145959</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FD22C07C-CA98-232F-528B-FE4FE0FDE179}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="617482" y="4703379"/>
+          <a:ext cx="4401164" cy="914528"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>65689</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>19707</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>409562</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>105630</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7DA41601-FC32-47D6-BB50-09781D4530C0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7692258" y="3015155"/>
+          <a:ext cx="4620270" cy="1419423"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>26276</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>183932</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>93885</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>165012</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagen 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8D1CD502-1F84-8C6D-8975-C4A2D22B23B2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7652845" y="4703380"/>
+          <a:ext cx="4344006" cy="933580"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -869,5 +1050,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Prueba con GRU nueva evaluada de forma distinta
</commit_message>
<xml_diff>
--- a/modelos_tfg/ResultadosCuantizacion.xlsx
+++ b/modelos_tfg/ResultadosCuantizacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6CC97AC-7020-403D-8D76-473D66869AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE5DBA64-C21D-4261-98B9-D784D8C0E729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -582,6 +582,270 @@
         <a:xfrm>
           <a:off x="7652845" y="4703380"/>
           <a:ext cx="4344006" cy="933580"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>94658</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>124811</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>100137</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Imagen 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2B63E0F2-EC44-1847-7741-7FE1B872D880}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="610914" y="5757106"/>
+          <a:ext cx="6529552" cy="1719979"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>43295</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>69272</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>672658</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>21826</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Imagen 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F23AA90D-0B9F-36E3-25B9-506FCBDA1A9E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="649431" y="10685317"/>
+          <a:ext cx="5106113" cy="1286054"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>34636</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>147205</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>470777</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>42575</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Imagen 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C7E07A7E-7001-1710-3D4B-30690559DC30}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="640772" y="9429750"/>
+          <a:ext cx="4220164" cy="1038370"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>34636</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>583159</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>47711</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Imagen 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8C3506C5-95C8-CF23-F60A-F6EE9653B9C9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="640772" y="8711045"/>
+          <a:ext cx="2886478" cy="619211"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>69272</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>165693</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>441613</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>58172</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Imagen 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B949DADF-4D22-2503-9938-801088CFC3D1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5844886" y="9448238"/>
+          <a:ext cx="4009159" cy="1035479"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>69273</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>77932</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>388311</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>97064</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Imagen 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0CECDD85-1CC7-BA26-967B-64F4A79247BB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5844887" y="8788977"/>
+          <a:ext cx="2743583" cy="590632"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>